<commit_message>
fixed eval 1 and 2
</commit_message>
<xml_diff>
--- a/Features.xlsx
+++ b/Features.xlsx
@@ -10,7 +10,7 @@
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="0" documentId="8_{E14E20CD-A1E0-4126-8471-DB0B58832913}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="43080" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{40574C69-72ED-4E2C-BD32-81F7BC54C045}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" xr2:uid="{40574C69-72ED-4E2C-BD32-81F7BC54C045}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -979,7 +979,7 @@
     <col min="4" max="4" width="36.9296875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="28.5">
+    <row r="1" spans="1:4">
       <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
@@ -1007,7 +1007,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="3" spans="1:4" ht="28.5">
+    <row r="3" spans="1:4">
       <c r="A3" s="4" t="s">
         <v>8</v>
       </c>
@@ -1021,7 +1021,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="4" spans="1:4" ht="42.75">
+    <row r="4" spans="1:4" ht="28.5">
       <c r="A4" s="4" t="s">
         <v>12</v>
       </c>
@@ -1049,7 +1049,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="6" spans="1:4" ht="57">
+    <row r="6" spans="1:4" ht="42.75">
       <c r="A6" s="4" t="s">
         <v>20</v>
       </c>
@@ -1063,7 +1063,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="7" spans="1:4" ht="57">
+    <row r="7" spans="1:4" ht="42.75">
       <c r="A7" s="4" t="s">
         <v>24</v>
       </c>
@@ -1077,7 +1077,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="8" spans="1:4" ht="57">
+    <row r="8" spans="1:4" ht="42.75">
       <c r="A8" s="4" t="s">
         <v>28</v>
       </c>
@@ -1119,7 +1119,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="11" spans="1:4" ht="57">
+    <row r="11" spans="1:4" ht="42.75">
       <c r="A11" s="4" t="s">
         <v>40</v>
       </c>
@@ -1133,7 +1133,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="12" spans="1:4" ht="71.25">
+    <row r="12" spans="1:4" ht="42.75">
       <c r="A12" s="4" t="s">
         <v>44</v>
       </c>
@@ -1147,7 +1147,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="13" spans="1:4" ht="57">
+    <row r="13" spans="1:4" ht="55.5">
       <c r="A13" s="4" t="s">
         <v>48</v>
       </c>
@@ -1189,7 +1189,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="16" spans="1:4" ht="71.25">
+    <row r="16" spans="1:4" ht="57">
       <c r="A16" s="4" t="s">
         <v>59</v>
       </c>

</xml_diff>